<commit_message>
Update live college audit and production trackers
</commit_message>
<xml_diff>
--- a/college-page-audit-dashboard.xlsx
+++ b/college-page-audit-dashboard.xlsx
@@ -614,7 +614,7 @@
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>2026-09-13 12:18:53 UTC</t>
+          <t>2026-09-13 16:34:08 UTC</t>
         </is>
       </c>
       <c r="C7" s="3" t="n"/>
@@ -3110,7 +3110,7 @@
     <row r="2">
       <c r="A2" s="3" t="inlineStr">
         <is>
-          <t>2026-09-13 12:18:53</t>
+          <t>2026-09-13 16:34:08</t>
         </is>
       </c>
       <c r="B2" s="3" t="inlineStr">
@@ -3142,7 +3142,7 @@
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>2026-09-13 12:18:53</t>
+          <t>2026-09-13 16:34:08</t>
         </is>
       </c>
       <c r="B3" s="3" t="inlineStr">
@@ -3174,7 +3174,7 @@
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>2026-09-13 12:18:53</t>
+          <t>2026-09-13 16:34:08</t>
         </is>
       </c>
       <c r="B4" s="3" t="inlineStr">
@@ -3206,7 +3206,7 @@
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>2026-09-13 12:18:53</t>
+          <t>2026-09-13 16:34:08</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
@@ -3238,7 +3238,7 @@
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
         <is>
-          <t>2026-09-13 12:18:53</t>
+          <t>2026-09-13 16:34:08</t>
         </is>
       </c>
       <c r="B6" s="3" t="inlineStr">
@@ -3270,7 +3270,7 @@
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
         <is>
-          <t>2026-09-13 12:18:53</t>
+          <t>2026-09-13 16:34:08</t>
         </is>
       </c>
       <c r="B7" s="3" t="inlineStr">
@@ -3302,7 +3302,7 @@
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
         <is>
-          <t>2026-09-13 12:18:53</t>
+          <t>2026-09-13 16:34:08</t>
         </is>
       </c>
       <c r="B8" s="3" t="inlineStr">
@@ -3334,7 +3334,7 @@
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
         <is>
-          <t>2026-09-13 12:18:53</t>
+          <t>2026-09-13 16:34:08</t>
         </is>
       </c>
       <c r="B9" s="3" t="inlineStr">
@@ -3366,7 +3366,7 @@
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
         <is>
-          <t>2026-09-13 12:18:53</t>
+          <t>2026-09-13 16:34:08</t>
         </is>
       </c>
       <c r="B10" s="3" t="inlineStr">
@@ -3398,7 +3398,7 @@
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
         <is>
-          <t>2026-09-13 12:18:53</t>
+          <t>2026-09-13 16:34:08</t>
         </is>
       </c>
       <c r="B11" s="3" t="inlineStr">
@@ -3430,7 +3430,7 @@
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
         <is>
-          <t>2026-09-13 12:18:53</t>
+          <t>2026-09-13 16:34:08</t>
         </is>
       </c>
       <c r="B12" s="3" t="inlineStr">
@@ -3462,7 +3462,7 @@
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
         <is>
-          <t>2026-09-13 12:18:53</t>
+          <t>2026-09-13 16:34:08</t>
         </is>
       </c>
       <c r="B13" s="3" t="inlineStr">
@@ -3494,7 +3494,7 @@
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
         <is>
-          <t>2026-09-13 12:18:53</t>
+          <t>2026-09-13 16:34:08</t>
         </is>
       </c>
       <c r="B14" s="3" t="inlineStr">
@@ -3526,7 +3526,7 @@
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
         <is>
-          <t>2026-09-13 12:18:53</t>
+          <t>2026-09-13 16:34:08</t>
         </is>
       </c>
       <c r="B15" s="3" t="inlineStr">
@@ -3558,7 +3558,7 @@
     <row r="16">
       <c r="A16" s="3" t="inlineStr">
         <is>
-          <t>2026-09-13 12:18:53</t>
+          <t>2026-09-13 16:34:08</t>
         </is>
       </c>
       <c r="B16" s="3" t="inlineStr">
@@ -3590,7 +3590,7 @@
     <row r="17">
       <c r="A17" s="3" t="inlineStr">
         <is>
-          <t>2026-09-13 12:18:53</t>
+          <t>2026-09-13 16:34:08</t>
         </is>
       </c>
       <c r="B17" s="3" t="inlineStr">
@@ -3622,7 +3622,7 @@
     <row r="18">
       <c r="A18" s="3" t="inlineStr">
         <is>
-          <t>2026-09-13 12:18:53</t>
+          <t>2026-09-13 16:34:08</t>
         </is>
       </c>
       <c r="B18" s="3" t="inlineStr">
@@ -3654,7 +3654,7 @@
     <row r="19">
       <c r="A19" s="3" t="inlineStr">
         <is>
-          <t>2026-09-13 12:18:53</t>
+          <t>2026-09-13 16:34:08</t>
         </is>
       </c>
       <c r="B19" s="3" t="inlineStr">
@@ -3686,7 +3686,7 @@
     <row r="20">
       <c r="A20" s="3" t="inlineStr">
         <is>
-          <t>2026-09-13 12:18:53</t>
+          <t>2026-09-13 16:34:08</t>
         </is>
       </c>
       <c r="B20" s="3" t="inlineStr">
@@ -3718,7 +3718,7 @@
     <row r="21">
       <c r="A21" s="3" t="inlineStr">
         <is>
-          <t>2026-09-13 12:18:53</t>
+          <t>2026-09-13 16:34:08</t>
         </is>
       </c>
       <c r="B21" s="3" t="inlineStr">
@@ -3750,7 +3750,7 @@
     <row r="22">
       <c r="A22" s="3" t="inlineStr">
         <is>
-          <t>2026-09-13 12:18:53</t>
+          <t>2026-09-13 16:34:08</t>
         </is>
       </c>
       <c r="B22" s="3" t="inlineStr">
@@ -3782,7 +3782,7 @@
     <row r="23">
       <c r="A23" s="3" t="inlineStr">
         <is>
-          <t>2026-09-13 12:18:53</t>
+          <t>2026-09-13 16:34:08</t>
         </is>
       </c>
       <c r="B23" s="3" t="inlineStr">
@@ -3814,7 +3814,7 @@
     <row r="24">
       <c r="A24" s="3" t="inlineStr">
         <is>
-          <t>2026-09-13 12:18:53</t>
+          <t>2026-09-13 16:34:08</t>
         </is>
       </c>
       <c r="B24" s="3" t="inlineStr">
@@ -3846,7 +3846,7 @@
     <row r="25">
       <c r="A25" s="3" t="inlineStr">
         <is>
-          <t>2026-09-13 12:18:53</t>
+          <t>2026-09-13 16:34:08</t>
         </is>
       </c>
       <c r="B25" s="3" t="inlineStr">

</xml_diff>